<commit_message>
adds total capital cost metric
</commit_message>
<xml_diff>
--- a/src/technology/small-modular-reactor/small-modular-reactor.xlsx
+++ b/src/technology/small-modular-reactor/small-modular-reactor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\small-modular-reactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C171F87-7AA2-4827-8500-3B3619B00F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4186DD4-F1DD-481B-806C-67F943E7250B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28050" yWindow="840" windowWidth="22965" windowHeight="19200" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="23730" yWindow="1155" windowWidth="27600" windowHeight="19515" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">designs!$A$1:$G$911</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indices!$A$1:$F$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indices!$A$1:$F$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">parameters!$A$1:$G$217</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1625" uniqueCount="152">
   <si>
     <t>Category</t>
   </si>
@@ -496,6 +496,15 @@
   </si>
   <si>
     <t>Ranges</t>
+  </si>
+  <si>
+    <t>USD/kWe</t>
+  </si>
+  <si>
+    <t>MWh/year</t>
+  </si>
+  <si>
+    <t>Total OCC</t>
   </si>
 </sst>
 </file>
@@ -847,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF3D170-DEC1-4938-B961-67DBF048922E}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -953,20 +962,34 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>100</v>
       </c>
-      <c r="D7">
+      <c r="D8">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F24">
-    <sortCondition ref="A3:A24"/>
-    <sortCondition ref="B3:B24"/>
-    <sortCondition ref="D3:D24"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F25">
+    <sortCondition ref="A3:A25"/>
+    <sortCondition ref="B3:B25"/>
+    <sortCondition ref="D3:D25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7908,7 +7931,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08421A62-7A7F-4754-940E-DE21752714F2}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -7943,6 +7966,9 @@
       <c r="C2" t="s">
         <v>28</v>
       </c>
+      <c r="D2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -7954,6 +7980,9 @@
       <c r="C3" t="s">
         <v>100</v>
       </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -7965,6 +7994,9 @@
       <c r="C4" t="s">
         <v>101</v>
       </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -7976,6 +8008,9 @@
       <c r="C5" t="s">
         <v>102</v>
       </c>
+      <c r="D5" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -7986,6 +8021,23 @@
       </c>
       <c r="C6" t="s">
         <v>103</v>
+      </c>
+      <c r="D6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tweaks BOAK Sensitivity plant number parameters; work in progress
</commit_message>
<xml_diff>
--- a/src/technology/small-modular-reactor/small-modular-reactor.xlsx
+++ b/src/technology/small-modular-reactor/small-modular-reactor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\small-modular-reactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4186DD4-F1DD-481B-806C-67F943E7250B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CC9164-BF00-4468-834E-1AB2E91DAE27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23730" yWindow="1155" windowWidth="27600" windowHeight="19515" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="20610" yWindow="975" windowWidth="28185" windowHeight="19515" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1625" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1624" uniqueCount="152">
   <si>
     <t>Category</t>
   </si>
@@ -2453,7 +2453,7 @@
     <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
     <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="58.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="81.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.28515625" bestFit="1" customWidth="1"/>
@@ -7073,7 +7073,7 @@
         <v>7</v>
       </c>
       <c r="E201">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F201" t="s">
         <v>72</v>
@@ -7234,7 +7234,7 @@
         <v>14</v>
       </c>
       <c r="E208">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F208" t="s">
         <v>72</v>
@@ -7256,8 +7256,8 @@
       <c r="D209">
         <v>15</v>
       </c>
-      <c r="E209" t="s">
-        <v>141</v>
+      <c r="E209">
+        <v>6</v>
       </c>
       <c r="F209" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
adds variable and fixed op and maint costs as metrics
</commit_message>
<xml_diff>
--- a/src/technology/small-modular-reactor/small-modular-reactor.xlsx
+++ b/src/technology/small-modular-reactor/small-modular-reactor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\small-modular-reactor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6256B30-DDC7-4616-A1D4-DC7E29F1FD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58FF924-531A-460B-8931-79D14348CE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2130" yWindow="465" windowWidth="31920" windowHeight="20805" tabRatio="778" activeTab="6" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="13125" windowHeight="18270" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2452" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="159">
   <si>
     <t>Category</t>
   </si>
@@ -520,6 +520,12 @@
   </si>
   <si>
     <t>BOAK 3 of 6 Orders</t>
+  </si>
+  <si>
+    <t>Variable Op and Maint</t>
+  </si>
+  <si>
+    <t>Fixed Op and Maint</t>
   </si>
 </sst>
 </file>
@@ -871,7 +877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF3D170-DEC1-4938-B961-67DBF048922E}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -991,12 +997,40 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C10" t="s">
         <v>97</v>
       </c>
-      <c r="D8">
+      <c r="D10">
         <v>0</v>
       </c>
     </row>
@@ -3542,7 +3576,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>39</v>
       </c>
@@ -3565,7 +3599,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -4094,7 +4128,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>39</v>
       </c>
@@ -4117,7 +4151,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>39</v>
       </c>
@@ -4163,7 +4197,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>39</v>
       </c>
@@ -4186,7 +4220,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>39</v>
       </c>
@@ -4209,7 +4243,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>39</v>
       </c>
@@ -4232,7 +4266,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>39</v>
       </c>
@@ -4255,7 +4289,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>39</v>
       </c>
@@ -4278,7 +4312,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>39</v>
       </c>
@@ -4301,7 +4335,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>39</v>
       </c>
@@ -4324,7 +4358,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>39</v>
       </c>
@@ -4347,7 +4381,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>39</v>
       </c>
@@ -4370,7 +4404,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>39</v>
       </c>
@@ -4393,7 +4427,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>39</v>
       </c>
@@ -4416,7 +4450,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>39</v>
       </c>
@@ -4439,7 +4473,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>39</v>
       </c>
@@ -4462,7 +4496,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>39</v>
       </c>
@@ -4485,7 +4519,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>39</v>
       </c>
@@ -4508,7 +4542,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>39</v>
       </c>
@@ -4531,7 +4565,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>39</v>
       </c>
@@ -4554,7 +4588,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>39</v>
       </c>
@@ -4577,7 +4611,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>39</v>
       </c>
@@ -4600,7 +4634,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>39</v>
       </c>
@@ -4623,7 +4657,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>39</v>
       </c>
@@ -4692,7 +4726,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>39</v>
       </c>
@@ -5198,7 +5232,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>39</v>
       </c>
@@ -5221,7 +5255,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>39</v>
       </c>
@@ -5750,7 +5784,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>39</v>
       </c>
@@ -5773,7 +5807,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>39</v>
       </c>
@@ -6302,7 +6336,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>39</v>
       </c>
@@ -6325,7 +6359,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>39</v>
       </c>
@@ -6854,7 +6888,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>39</v>
       </c>
@@ -6877,7 +6911,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>39</v>
       </c>
@@ -7406,7 +7440,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>39</v>
       </c>
@@ -7429,7 +7463,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>39</v>
       </c>
@@ -7958,7 +7992,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>39</v>
       </c>
@@ -7981,7 +8015,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>39</v>
       </c>
@@ -8027,7 +8061,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>39</v>
       </c>
@@ -8050,7 +8084,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>39</v>
       </c>
@@ -8073,7 +8107,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>39</v>
       </c>
@@ -8096,7 +8130,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>39</v>
       </c>
@@ -8119,7 +8153,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>39</v>
       </c>
@@ -8142,7 +8176,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>39</v>
       </c>
@@ -8165,7 +8199,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>39</v>
       </c>
@@ -8188,7 +8222,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>39</v>
       </c>
@@ -8211,7 +8245,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>39</v>
       </c>
@@ -8234,7 +8268,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>39</v>
       </c>
@@ -8257,7 +8291,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>39</v>
       </c>
@@ -8280,7 +8314,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>39</v>
       </c>
@@ -8303,7 +8337,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>39</v>
       </c>
@@ -8326,7 +8360,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>39</v>
       </c>
@@ -8349,7 +8383,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>39</v>
       </c>
@@ -8372,7 +8406,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>39</v>
       </c>
@@ -8395,7 +8429,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>39</v>
       </c>
@@ -8418,7 +8452,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>39</v>
       </c>
@@ -8441,7 +8475,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>39</v>
       </c>
@@ -8464,7 +8498,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>39</v>
       </c>
@@ -8487,7 +8521,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>39</v>
       </c>
@@ -8556,7 +8590,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>39</v>
       </c>
@@ -8579,7 +8613,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>39</v>
       </c>
@@ -8602,7 +8636,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>39</v>
       </c>
@@ -8625,7 +8659,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>39</v>
       </c>
@@ -8648,7 +8682,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>39</v>
       </c>
@@ -8671,7 +8705,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>39</v>
       </c>
@@ -8694,7 +8728,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>39</v>
       </c>
@@ -8717,7 +8751,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>39</v>
       </c>
@@ -8740,7 +8774,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>39</v>
       </c>
@@ -8763,7 +8797,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>39</v>
       </c>
@@ -8786,7 +8820,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>39</v>
       </c>
@@ -8809,7 +8843,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>39</v>
       </c>
@@ -8832,7 +8866,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>39</v>
       </c>
@@ -8855,7 +8889,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>39</v>
       </c>
@@ -8878,7 +8912,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>39</v>
       </c>
@@ -8901,7 +8935,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>39</v>
       </c>
@@ -8924,7 +8958,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>39</v>
       </c>
@@ -8947,7 +8981,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>39</v>
       </c>
@@ -8970,7 +9004,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>39</v>
       </c>
@@ -8993,7 +9027,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>39</v>
       </c>
@@ -9016,7 +9050,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>39</v>
       </c>
@@ -9039,7 +9073,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>39</v>
       </c>
@@ -9108,7 +9142,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>39</v>
       </c>
@@ -9131,7 +9165,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>39</v>
       </c>
@@ -9154,7 +9188,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>39</v>
       </c>
@@ -9177,7 +9211,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>39</v>
       </c>
@@ -9200,7 +9234,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>39</v>
       </c>
@@ -9223,7 +9257,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>39</v>
       </c>
@@ -9246,7 +9280,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>39</v>
       </c>
@@ -9269,7 +9303,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>39</v>
       </c>
@@ -9292,7 +9326,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>39</v>
       </c>
@@ -9315,7 +9349,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>39</v>
       </c>
@@ -9338,7 +9372,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>39</v>
       </c>
@@ -9361,7 +9395,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>39</v>
       </c>
@@ -9384,7 +9418,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>39</v>
       </c>
@@ -9407,7 +9441,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>39</v>
       </c>
@@ -9430,7 +9464,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>39</v>
       </c>
@@ -9453,7 +9487,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>39</v>
       </c>
@@ -9476,7 +9510,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>39</v>
       </c>
@@ -9499,7 +9533,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>39</v>
       </c>
@@ -9522,7 +9556,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>39</v>
       </c>
@@ -9545,7 +9579,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>39</v>
       </c>
@@ -9568,7 +9602,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>39</v>
       </c>
@@ -9591,7 +9625,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>39</v>
       </c>
@@ -9660,7 +9694,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>39</v>
       </c>
@@ -9683,7 +9717,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>39</v>
       </c>
@@ -9706,7 +9740,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>39</v>
       </c>
@@ -9729,7 +9763,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>39</v>
       </c>
@@ -9752,7 +9786,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>39</v>
       </c>
@@ -9775,7 +9809,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>39</v>
       </c>
@@ -9798,7 +9832,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>39</v>
       </c>
@@ -9821,7 +9855,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>39</v>
       </c>
@@ -9844,7 +9878,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>39</v>
       </c>
@@ -9867,7 +9901,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>39</v>
       </c>
@@ -9890,7 +9924,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>39</v>
       </c>
@@ -9913,7 +9947,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>39</v>
       </c>
@@ -9936,7 +9970,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>39</v>
       </c>
@@ -9959,7 +9993,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>39</v>
       </c>
@@ -9982,7 +10016,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>39</v>
       </c>
@@ -10005,7 +10039,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>39</v>
       </c>
@@ -10028,7 +10062,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>39</v>
       </c>
@@ -10051,7 +10085,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>39</v>
       </c>
@@ -10074,7 +10108,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>39</v>
       </c>
@@ -10097,7 +10131,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>39</v>
       </c>
@@ -10120,7 +10154,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>39</v>
       </c>
@@ -10143,7 +10177,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>39</v>
       </c>
@@ -10212,7 +10246,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>39</v>
       </c>
@@ -10237,13 +10271,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G313" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}">
-    <filterColumn colId="1">
+    <filterColumn colId="2">
       <filters>
-        <filter val="BOAK 2 of 6 Orders"/>
-        <filter val="BOAK 3 of 6 Orders"/>
-        <filter val="BOAK 4 of 6 Orders"/>
-        <filter val="BOAK 5 of 6 Orders"/>
-        <filter val="BOAK 6 Orders"/>
+        <filter val="om_fixed"/>
+        <filter val="om_variable"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -10259,7 +10290,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08421A62-7A7F-4754-940E-DE21752714F2}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -10366,6 +10397,28 @@
       </c>
       <c r="D7" t="s">
         <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>